<commit_message>
Fix P/E benchmark: prefer own 5yr history over sector peer median
Root cause: _t_val() used min(hist_avg, sect_med) as the P/E benchmark.
For quality compounders with a structural sector premium (MSFT: 5yr avg
33.9x vs Software peers 19.1x), the peer median became the binding
constraint — making MSFT forward P/E 24.8x look +30% expensive → tier LOW,
despite being -27% below its own history.

Fix: use own 5-year average as primary benchmark (sector median as fallback
when history is unavailable). Cap hist_avg at 50x to exclude ZIRP/bubble-era
distortion (AMD 123x, DIS 66x) — preserving company-specific signal without
rewarding bubble-era multiples.

MSFT result: tier_pe LOW→HIGH, score_pe 3.8→9.9, auto_score 6.3→7.8
AMD: tier_pe LOW (unchanged in effective result; P/E data sparse this run)

Also: add sector_pe_med to scorecard_metrics dict for diagnostics.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/excel/MSFT_model.xlsx
+++ b/static/excel/MSFT_model.xlsx
@@ -7344,11 +7344,11 @@
         </is>
       </c>
       <c r="B5" s="43" t="n">
-        <v>3109317.9451</v>
+        <v>3089558.3213</v>
       </c>
       <c r="C5" s="44" t="inlineStr">
         <is>
-          <t>FMP marketCap  |  price $418.57</t>
+          <t>FMP marketCap  |  price $415.91</t>
         </is>
       </c>
     </row>
@@ -7659,25 +7659,27 @@
       </c>
       <c r="B32" s="53" t="inlineStr">
         <is>
-          <t>Not available</t>
+          <t>AAA</t>
         </is>
       </c>
       <c r="C32" s="44" t="inlineStr">
         <is>
-          <t>FMP /ratings endpoint</t>
+          <t>User input</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>FRED matched yield</t>
-        </is>
-      </c>
-      <c r="B33" s="53" t="n"/>
+          <t>FRED matched yield  (rating-tier index)</t>
+        </is>
+      </c>
+      <c r="B33" s="46" t="n">
+        <v>0.0507</v>
+      </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
-          <t>No rating returned — FRED method not applicable</t>
+          <t>FRED BAMLC0A1CAAAEY — AAA</t>
         </is>
       </c>
     </row>
@@ -7767,7 +7769,7 @@
       </c>
       <c r="C39" s="49" t="inlineStr">
         <is>
-          <t>Default = average of 2 source(s) above — override freely</t>
+          <t>Default = average of 3 source(s) above — override freely</t>
         </is>
       </c>
     </row>
@@ -9982,7 +9984,7 @@
         </is>
       </c>
       <c r="B61" s="111" t="n">
-        <v>418.57</v>
+        <v>415.91</v>
       </c>
       <c r="C61" s="103" t="n"/>
       <c r="D61" s="103" t="n"/>
@@ -10082,7 +10084,7 @@
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="113" t="inlineStr">
         <is>
-          <t>JS SCORECARD — MSFT  |  Master Prompt v2  |  25 May 2026  |  Sector bucket: Tech Growth</t>
+          <t>JS SCORECARD — MSFT  |  Master Prompt v2  |  27 May 2026  |  Sector bucket: Tech Growth</t>
         </is>
       </c>
     </row>
@@ -10599,16 +10601,16 @@
       </c>
       <c r="D22" s="129" t="inlineStr">
         <is>
-          <t>Current 36.3x  |  5yr avg 33.9x  |  Sector median 19.1x  |  DCF-implied 29.0x [ref only — not used as benchmark]  [+90% vs benchmark]  [trail=0.00 | fwd_pe=24.9x→2.36 | abs=1.5 → blended 40/40/20=1.24]  PEG=110.76 (fwd_pe=24.9x / eps_growth=22%)  [revision:Strong upgrade cycle→+0.50]</t>
-        </is>
-      </c>
-      <c r="E22" s="136" t="inlineStr">
-        <is>
-          <t>LOW</t>
+          <t>Fwd P/E 24.8x (scoring basis)  |  5yr avg 33.9x  |  Sector median 19.1x  |  DCF-implied 29.0x [ref only — not used as benchmark]  [-27% vs benchmark]  [trail=10.00 | fwd_pe=24.8x→10.00 | abs=7.0 → blended 40/40/20=9.40]  PEG=110.32 (fwd_pe=24.8x / eps_growth=22%)  [revision:Strong upgrade cycle→+0.50]</t>
+        </is>
+      </c>
+      <c r="E22" s="135" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="F22" s="131" t="n">
-        <v>1.74</v>
+        <v>9.9</v>
       </c>
       <c r="G22" s="132">
         <f>IF(F22="",0,C22*F22*10)</f>
@@ -10616,7 +10618,7 @@
       </c>
       <c r="H22" s="133" t="inlineStr">
         <is>
-          <t>Current 36.3x  |  5yr avg 33.9x  |  Sector median 19.1x  |  DCF-implied 29.0x [ref only — not used as benchmark]  [+90% vs benchmark]  [trail=0.00 | fwd_pe=24.9x→2.36 | abs=1.5 → blended 40/40/20=1.24]  PEG=110.76 (fwd_pe=24.9x / eps_growth=22%)  [revision:Strong upgrade cycle→+0.50]</t>
+          <t>Fwd P/E 24.8x (scoring basis)  |  5yr avg 33.9x  |  Sector median 19.1x  |  DCF-implied 29.0x [ref only — not used as benchmark]  [-27% vs benchmark]  [trail=10.00 | fwd_pe=24.8x→10.00 | abs=7.0 → blended 40/40/20=9.40]  PEG=110.32 (fwd_pe=24.8x / eps_growth=22%)  [revision:Strong upgrade cycle→+0.50]</t>
         </is>
       </c>
     </row>
@@ -10636,7 +10638,7 @@
       </c>
       <c r="D23" s="129" t="inlineStr">
         <is>
-          <t>Current 51.6x  |  5yr avg 41.2x  |  Sector median 13.8x  |  DCF-implied 41.3x [ref only — not used as benchmark]  [+274% vs benchmark]  [trail=0.00 | fwd_pfcf=37.2x→0.00 | abs=1.5 → blended 40/40/20=0.30]  [fcf_yield=1.9% vs rf=4.6%  spread=-2.6%→modifier=-0.50]</t>
+          <t>Current 51.6x  |  5yr avg 41.2x  |  Sector median 13.8x  |  DCF-implied 41.3x [ref only — not used as benchmark]  [+25% vs benchmark]  [trail=2.97 | fwd_pfcf=36.9x→8.57 | abs=1.5 → blended 40/40/20=4.91]  [fcf_yield=1.9% vs rf=4.6%  spread=-2.6%→modifier=-0.50]</t>
         </is>
       </c>
       <c r="E23" s="136" t="inlineStr">
@@ -10645,7 +10647,7 @@
         </is>
       </c>
       <c r="F23" s="131" t="n">
-        <v>0</v>
+        <v>4.41</v>
       </c>
       <c r="G23" s="132">
         <f>IF(F23="",0,C23*F23*10)</f>
@@ -10653,7 +10655,7 @@
       </c>
       <c r="H23" s="133" t="inlineStr">
         <is>
-          <t>Current 51.6x  |  5yr avg 41.2x  |  Sector median 13.8x  |  DCF-implied 41.3x [ref only — not used as benchmark]  [+274% vs benchmark]  [trail=0.00 | fwd_pfcf=37.2x→0.00 | abs=1.5 → blended 40/40/20=0.30]  [fcf_yield=1.9% vs rf=4.6%  spread=-2.6%→modifier=-0.50]</t>
+          <t>Current 51.6x  |  5yr avg 41.2x  |  Sector median 13.8x  |  DCF-implied 41.3x [ref only — not used as benchmark]  [+25% vs benchmark]  [trail=2.97 | fwd_pfcf=36.9x→8.57 | abs=1.5 → blended 40/40/20=4.91]  [fcf_yield=1.9% vs rf=4.6%  spread=-2.6%→modifier=-0.50]</t>
         </is>
       </c>
     </row>

</xml_diff>